<commit_message>
feat: Week 2026-W40 — new skills batch
</commit_message>
<xml_diff>
--- a/spreadsheets/Claude_Skills_Week_2026-W40.xlsx
+++ b/spreadsheets/Claude_Skills_Week_2026-W40.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Professional / Domain-Specific</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Legal Domain Advisor</t>
+          <t>Legal Domain Assistant</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -583,12 +583,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>404kidwiz--csharp-developer</t>
+          <t>aiskillstore--python-style-guide</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>C# Developer (404kidwiz)</t>
+          <t>Python Style Guide Assistant</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -606,34 +606,34 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://smithery.ai/skills/404kidwiz/csharp-developer</t>
+          <t>https://smithery.ai/skills/aiskillstore/python-style-guide</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>404kidwiz--csharp-developer.md</t>
+          <t>aiskillstore--python-style-guide.md</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Everyday Household / Busy Family</t>
+          <t>Software Development by Language</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Family &amp; Home</t>
+          <t>Software Development</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>openclaw--withings-family</t>
+          <t>404kidwiz--csharp-developer</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Withings Family Health Assistant</t>
+          <t>C# Developer Assistant</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -641,9 +641,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
@@ -651,55 +651,100 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://smithery.ai/skills/openclaw/withings-family</t>
+          <t>https://smithery.ai/skills/404kidwiz/csharp-developer</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>openclaw--withings-family.md</t>
+          <t>404kidwiz--csharp-developer.md</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Everyday Household / Busy Family</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Everyday Household</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>openclaw--withings-family</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Withings Family Health Assistant</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://smithery.ai/skills/openclaw/withings-family</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>openclaw--withings-family.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>New Claude Features &amp; Hooks</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Agent Frameworks</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Developer Tools</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>ECC-Antigravity</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>ECC Antigravity — Claude Code Runtime &amp; Lifecycle Hooks</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ECC-Antigravity Runtime</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://github.com/cloudblower/ECC-Antigravity</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>ecc-antigravity.md</t>
         </is>

</xml_diff>